<commit_message>
103th Commit: Epic Two Completed
</commit_message>
<xml_diff>
--- a/EPIC_0002_Driver_Onboarding.xlsx
+++ b/EPIC_0002_Driver_Onboarding.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EFD7B87-C5F7-4FDA-B530-E8F52547ACCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43A87AE-9132-4847-BFED-D888199A1F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="31">
   <si>
     <t>Requirement Title</t>
   </si>
@@ -554,6 +554,140 @@
   </si>
   <si>
     <t>Admin Web portal is accessible</t>
+  </si>
+  <si>
+    <t>1. Reload User App Completely,reload_app,user,
+2. Reload Driver App Completely,reload_app,driver,
+3. Load Driver App,switch_to,driver,
+4. Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+5. Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+6. Click Agree,tap,,"mobile.driver.agree.btn"
+7. Click Get Started,tap,,"mobile.driver.get_started.btn"
+8. Click Next,tap,,"mobile.driver.next.btn"
+9. Click Mobile Number Button,tap,,"mobile.customer.mobile_number_field.btn"
+10. Click Close,tap_if_present,,"mobile.driver.cancel.btn"
+11. Enter Mobile Number,type,{randomPhone}&gt;&gt;driverNumber,"mobile.driver.edit_text.input"
+12.Wait For Continue,wait_until_visible,,"mobile.driver.continue.btn"
+13.Click on Continue,tap,,"mobile.driver.continue.btn"
+14. wait for OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+15. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+16. Wait for Finish,wait_until_visible,,"mobile.driver.finish.btn"
+17. Click on Finish,tap,"mobile.driver.finish.btn"
+18.Wait For Profile Registation Page,wait_until_visible,"mobile.driver.Register.profile.pen_icon"
+19.Click on ProfileImage,tap,,"mobile.driver.Register.profile.pen_icon"
+20.Wait For Camera,wait_until_visible,"mobile.driver.Camera.btn"
+21.Click on camera,tap,,"mobile.driver.Camera.btn"
+22.Click while using this app Notification,tap,,"mobile.driver.camera_allow.btn"
+23.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+24.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+25.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+26.Type Driver Name,type,autoDriver{randomAlpha}&gt;&gt;driverName,"mobile.driver.driver_name_input"
+27.Wait For Keyboard Minimises,hide_keyboard,,
+28.Enter Whatsapp Number,type,{randomPhone}&gt;&gt;whatsappNumber,"mobile.driver.whatsapp_no.input_box"
+29.Enter Email,type,{driverName}@gmail.com&gt;&gt;driverEmail,"mobile.driver.driver_email_input"
+30.Wait For Keyboard Minimises,hide_keyboard,,
+31.Click  Gender Box Male,tap,,"mobile.driver.select_gender_male"
+32.Scroll Screen,swipe,up,
+33.Click  Social Media,tap,,"mobile.driver.how_did_you_hear_about_us"
+34.Select Instagram,tap,,"mobile.driver.select_option_instagram"
+35.Click Terms And Conditions,tap_coordinate ,124:1758,COORDINATE_MODE
+36.Click Sign Up,tap,,"mobile.driver.sign_up_btn"
+37.Wait For Vehicle Type,wait_until_visible,"mobile.driver.Service_vehicle_Type_heading"
+38.Select Auto Ride,tap,,"mobile.driver.select_auto_ride"
+39.Click Next,tap,,"mobile.driver.auto_ride_next_btn"
+40.Wait for Pop Up,wait_if_present,,"mobile.driver.driver_location_allow.btn"
+41.Click While Using This App Notification,tap_if_present,,"mobile.driver.driver_location_allow.btn"
+42.Click Upload image Icon,tap,,"mobile.driver.vehicle_image_upload_icon"
+43.Click on camera,tap,,"mobile.driver.Camera.btn"
+44.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+45.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+46.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+47.Click Select Vehicle Type Dropdown,tap,,"mobile.driver.vehicle_type_dropdown"
+48.Select Option Pink Auto,tap,,"mobile.driver.vehicle_type_option.pink_auto"
+49.Type Model Name,type,petrol,"mobile.driver.vehicle_model_name.input_box"
+50.Click Vehicle Model Year,tap,,"mobile.driver.vehicle_type_model_year.dropdown"
+51.Select Year,tap,,"mobile.driver.vehicle_type_model_year.option_year"
+52..Type Vehicle Plate No,type,TN22CL5170,"mobile.driver.Vehicle_plate_number"
+53.Click the Seat Number,tap,,"mobile.driver.select_seat_number.drop_down"
+54.Select Number Of Seat,tap,"mobile.driver.select_seat_number.option_three"
+55.Scroll Screen,swipe,up,
+56.Type Vehicle Color,type,Pink,"mobile.driver.Vehicle_colour"
+57.Save Vehicle Detaills,tap,,"mobile.drivers_vehicle_details.save_btn"
+58. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+59. Click Upload,tap,,"mobile.driver.upload.btn"
+60. Upload License,tap,,"mobile.driver.upload_docs.btn"
+61.Click on camera,tap,,"mobile.driver.Camera.btn"
+62.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+63.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+64.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+65. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+66. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+67. Click Month,tap,,"mobile.driver.next_month.btn"
+68. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+69. Click Ok,tap,,"mobile.driver.ok.btn"
+70. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+71.Click Next Button,tap,,"mobile.drivers.after_upload_doc.next_btn"
+72.Enter Account Holder,type,{driverName},"mobile.driver.bank_details.account_holder_name"
+73.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+74.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+75.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+76.Wait For Keyboard Minimises,hide_keyboard,,
+77.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
+78.Wait For Keyboard Minimises,hide_keyboard,,
+79.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+80.Wait For Logout,wait_until_visible,"mobile.drivers.after_upload_doc.logout_btn"
+81.Click Logout,tap,,"mobile.drivers.after_upload_doc.logout_btn"
+82.Click Confirm Logout,tap,,"mobile.drivers.after_upload_doc.logout_confirm_btn"
+83.Reload Driver App Completely,reload_app,driver,
+84.Load Admin App,switch_to,web,
+85.Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+87.Click drivers menu,click,,"admin.drivers.menu.icon"
+88.Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+89.Filter by Name,type,{driverName},"admin.drivers.name_filter.input"
+90.Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+91. Click Doc Icon,click,,"admin.drivers.docs.icon"
+92. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
+93. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+94. Click Approve Driver,click,,"admin.drivers.docs.approval"
+95. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
+96. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+97. Click drivers menu,click,,"admin.drivers.menu.icon"
+98. Click UnApproved Drivers,click,,"admin.drivers.unapproved_docs.link"
+99.Wait For load,wait,3000,
+100.Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
+101.Scroll Grid,tab,10,"admin.drivers.name_filter.input"
+102.Click Eye Icon,click,,"admin.drivers.unapproved_driver.eye_icon"
+103.Wait For Data,wait,3000,
+104.Click Close Button,click,,"admin.drivers.unapproved_driver.eye_icon.close_btn"
+105.Click ThumbsUp For Approve,click,,"admin.drivers.unapproved_driver.thumbs_up"
+106.Wait For Toast,wait,3000,
+107. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+108.Click drivers menu,click,,"admin.drivers.menu.icon"
+109.Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+110.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
+111. Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
+112.Load Driver App,switch_to,driver,
+113.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+114.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+115.Click Agree,tap,,"mobile.driver.agree.btn"
+116.Click Get Started,tap,,"mobile.driver.get_started.btn"
+117.Click Next,tap,,"mobile.driver.next.btn"
+118.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+119.Click Close,tap,,"mobile.driver.cancel.btn"
+120.Enter Mobile Number,type,{driverNumber},"mobile.driver.edit_text.input"
+121.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+122.Click Continue,tap,,"mobile.driver.continue.btn"
+123.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+124.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+125.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+126.Wait For Pageload,wait,3000,
+127. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+128. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+129. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+130. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+131. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+132. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"</t>
   </si>
 </sst>
 </file>
@@ -1008,8 +1142,8 @@
     <col min="6" max="6" width="45.77734375" customWidth="1"/>
     <col min="7" max="7" width="71.44140625" customWidth="1"/>
     <col min="8" max="8" width="40.44140625" customWidth="1"/>
-    <col min="9" max="9" width="61.88671875" customWidth="1"/>
-    <col min="10" max="10" width="32.88671875" customWidth="1"/>
+    <col min="9" max="9" width="41.6640625" customWidth="1"/>
+    <col min="10" max="10" width="53.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1064,7 +1198,7 @@
         <v>28</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
@@ -1072,7 +1206,9 @@
       <c r="I2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="J2" s="2"/>
+      <c r="J2" s="2" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>

</xml_diff>

<commit_message>
104th Commit: Epic Two Updated Driver Signup Page Lag Fixed
</commit_message>
<xml_diff>
--- a/EPIC_0002_Driver_Onboarding.xlsx
+++ b/EPIC_0002_Driver_Onboarding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B43A87AE-9132-4847-BFED-D888199A1F7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D11E450-966B-4F26-B836-A88833BBF920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -582,112 +582,110 @@
 24.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
 25.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
 26.Type Driver Name,type,autoDriver{randomAlpha}&gt;&gt;driverName,"mobile.driver.driver_name_input"
-27.Wait For Keyboard Minimises,hide_keyboard,,
-28.Enter Whatsapp Number,type,{randomPhone}&gt;&gt;whatsappNumber,"mobile.driver.whatsapp_no.input_box"
-29.Enter Email,type,{driverName}@gmail.com&gt;&gt;driverEmail,"mobile.driver.driver_email_input"
-30.Wait For Keyboard Minimises,hide_keyboard,,
-31.Click  Gender Box Male,tap,,"mobile.driver.select_gender_male"
-32.Scroll Screen,swipe,up,
-33.Click  Social Media,tap,,"mobile.driver.how_did_you_hear_about_us"
-34.Select Instagram,tap,,"mobile.driver.select_option_instagram"
-35.Click Terms And Conditions,tap_coordinate ,124:1758,COORDINATE_MODE
-36.Click Sign Up,tap,,"mobile.driver.sign_up_btn"
-37.Wait For Vehicle Type,wait_until_visible,"mobile.driver.Service_vehicle_Type_heading"
-38.Select Auto Ride,tap,,"mobile.driver.select_auto_ride"
-39.Click Next,tap,,"mobile.driver.auto_ride_next_btn"
-40.Wait for Pop Up,wait_if_present,,"mobile.driver.driver_location_allow.btn"
-41.Click While Using This App Notification,tap_if_present,,"mobile.driver.driver_location_allow.btn"
-42.Click Upload image Icon,tap,,"mobile.driver.vehicle_image_upload_icon"
-43.Click on camera,tap,,"mobile.driver.Camera.btn"
-44.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
-45.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
-46.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
-47.Click Select Vehicle Type Dropdown,tap,,"mobile.driver.vehicle_type_dropdown"
-48.Select Option Pink Auto,tap,,"mobile.driver.vehicle_type_option.pink_auto"
-49.Type Model Name,type,petrol,"mobile.driver.vehicle_model_name.input_box"
-50.Click Vehicle Model Year,tap,,"mobile.driver.vehicle_type_model_year.dropdown"
-51.Select Year,tap,,"mobile.driver.vehicle_type_model_year.option_year"
-52..Type Vehicle Plate No,type,TN22CL5170,"mobile.driver.Vehicle_plate_number"
-53.Click the Seat Number,tap,,"mobile.driver.select_seat_number.drop_down"
-54.Select Number Of Seat,tap,"mobile.driver.select_seat_number.option_three"
-55.Scroll Screen,swipe,up,
-56.Type Vehicle Color,type,Pink,"mobile.driver.Vehicle_colour"
-57.Save Vehicle Detaills,tap,,"mobile.drivers_vehicle_details.save_btn"
-58. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
-59. Click Upload,tap,,"mobile.driver.upload.btn"
-60. Upload License,tap,,"mobile.driver.upload_docs.btn"
-61.Click on camera,tap,,"mobile.driver.Camera.btn"
-62.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
-63.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
-64.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
-65. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
-66. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
-67. Click Month,tap,,"mobile.driver.next_month.btn"
-68. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
-69. Click Ok,tap,,"mobile.driver.ok.btn"
-70. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
-71.Click Next Button,tap,,"mobile.drivers.after_upload_doc.next_btn"
-72.Enter Account Holder,type,{driverName},"mobile.driver.bank_details.account_holder_name"
-73.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
-74.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
-75.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+27.Enter Whatsapp Number,type,{randomPhone}&gt;&gt;whatsappNumber,"mobile.driver.whatsapp_no.input_box"
+28.Enter Email,type,{driverName}@gmail.com&gt;&gt;driverEmail,"mobile.driver.driver_email_input"
+29.Click  Gender Box Male,tap,,"mobile.driver.select_gender_male"
+30.Scroll Screen,swipe,up,
+31.Click  Social Media,tap,,"mobile.driver.how_did_you_hear_about_us"
+32.Select Instagram,tap,,"mobile.driver.select_option_instagram"
+33.Click Terms And Conditions,tap_coordinate ,124:1758,COORDINATE_MODE
+34.Click Sign Up,tap,,"mobile.driver.sign_up_btn"
+35.Wait For Vehicle Type,wait_until_visible,"mobile.driver.Service_vehicle_Type_heading"
+36.Select Auto Ride,tap,,"mobile.driver.select_auto_ride"
+37.Click Next,tap,,"mobile.driver.auto_ride_next_btn"
+38.Wait for Pop Up,wait_if_present,,"mobile.driver.driver_location_allow.btn"
+39.Click While Using This App Notification,tap_if_present,,"mobile.driver.driver_location_allow.btn"
+40.Click Upload image Icon,tap,,"mobile.driver.vehicle_image_upload_icon"
+41.Click on camera,tap,,"mobile.driver.Camera.btn"
+42.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+43.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+44.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+45.Click Select Vehicle Type Dropdown,tap,,"mobile.driver.vehicle_type_dropdown"
+46.Select Option Pink Auto,tap,,"mobile.driver.vehicle_type_option.pink_auto"
+47.Type Model Name,type,petrol,"mobile.driver.vehicle_model_name.input_box"
+48.Click Vehicle Model Year,tap,,"mobile.driver.vehicle_type_model_year.dropdown"
+49.Select Year,tap,,"mobile.driver.vehicle_type_model_year.option_year"
+50.Type Vehicle Plate No,type,TN22CL5170,"mobile.driver.Vehicle_plate_number"
+51.Click the Seat Number,tap,,"mobile.driver.select_seat_number.drop_down"
+52.Select Number Of Seat,tap,"mobile.driver.select_seat_number.option_three"
+53.Scroll Screen,swipe,up,
+54.Type Vehicle Color,type,Pink,"mobile.driver.Vehicle_colour"
+55.Save Vehicle Detaills,tap,,"mobile.drivers_vehicle_details.save_btn"
+56. Wait For Upload,wait_until_visible,,"mobile.driver.upload.btn"
+57. Click Upload,tap,,"mobile.driver.upload.btn"
+58. Upload License,tap,,"mobile.driver.upload_docs.btn"
+59.Click on camera,tap,,"mobile.driver.Camera.btn"
+60.Click on Camera Icon,tap,,"mobile.driver.camera_selfie.btn"
+61.Click on Select Image,tap,,"mobile.driver.selfie_select.btn"
+62.Click on Crop Button,tap,,"mobile.driver.selfie_crop.btn"
+63. Wait For Add Document,wait_until_visible,,"mobile.driver.add_documents.header"
+64. Click Calendar,tap_coordinate,121:1539,COORDINATE_MODE
+65. Click Month,tap,,"mobile.driver.next_month.btn"
+66. Click Date,tap_coordinate,943:1290,COORDINATE_MODE
+67. Click Ok,tap,,"mobile.driver.ok.btn"
+68. Click Upload Submission,tap,,"mobile.driver.upload_docs.btn"
+69.Click Next Button,tap,,"mobile.drivers.after_upload_doc.next_btn"
+70.Enter Account Holder,type,{driverName},"mobile.driver.bank_details.account_holder_name"
+71.Enter Account Number,type,50100123456789,"mobile.driver.bank_details.account_number"
+72.Enter Confirm Account Number,type,50100123456789,"mobile.driver.bank_details.confirm_account_number"
+73.Enter IFSC Code,type,HDFC0001234,"mobile.driver.bank_details.confirm_ifsc_code"
+74.Wait For Keyboard Minimises,hide_keyboard,,
+75.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
 76.Wait For Keyboard Minimises,hide_keyboard,,
-77.Enter Upi Id,type,sujanpariyar07@fam,"mobile.driver.bank_details.upi_id"
-78.Wait For Keyboard Minimises,hide_keyboard,,
-79.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
-80.Wait For Logout,wait_until_visible,"mobile.drivers.after_upload_doc.logout_btn"
-81.Click Logout,tap,,"mobile.drivers.after_upload_doc.logout_btn"
-82.Click Confirm Logout,tap,,"mobile.drivers.after_upload_doc.logout_confirm_btn"
-83.Reload Driver App Completely,reload_app,driver,
-84.Load Admin App,switch_to,web,
-85.Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
-86.Click Dashboard Icon,click,,"web.global.menu.dashboard"
-87.Click drivers menu,click,,"admin.drivers.menu.icon"
-88.Click Pending Documents,click,,"admin.drivers.pending_docs.link"
-89.Filter by Name,type,{driverName},"admin.drivers.name_filter.input"
-90.Scroll Grid,tab,7,"admin.drivers.name_filter.input"
-91. Click Doc Icon,click,,"admin.drivers.docs.icon"
-92. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
-93. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
-94. Click Approve Driver,click,,"admin.drivers.docs.approval"
-95. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
-96. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-97. Click drivers menu,click,,"admin.drivers.menu.icon"
-98. Click UnApproved Drivers,click,,"admin.drivers.unapproved_docs.link"
-99.Wait For load,wait,3000,
-100.Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
-101.Scroll Grid,tab,10,"admin.drivers.name_filter.input"
-102.Click Eye Icon,click,,"admin.drivers.unapproved_driver.eye_icon"
-103.Wait For Data,wait,3000,
-104.Click Close Button,click,,"admin.drivers.unapproved_driver.eye_icon.close_btn"
-105.Click ThumbsUp For Approve,click,,"admin.drivers.unapproved_driver.thumbs_up"
-106.Wait For Toast,wait,3000,
-107. Click Dashboard Icon,click,,"web.global.menu.dashboard"
-108.Click drivers menu,click,,"admin.drivers.menu.icon"
-109.Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
-110.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
-111. Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
-112.Load Driver App,switch_to,driver,
-113.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
-114.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
-115.Click Agree,tap,,"mobile.driver.agree.btn"
-116.Click Get Started,tap,,"mobile.driver.get_started.btn"
-117.Click Next,tap,,"mobile.driver.next.btn"
-118.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
-119.Click Close,tap,,"mobile.driver.cancel.btn"
-120.Enter Mobile Number,type,{driverNumber},"mobile.driver.edit_text.input"
-121.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
-122.Click Continue,tap,,"mobile.driver.continue.btn"
-123.Enter OTP,type,123456,"mobile.driver.edit_text.input"
-124.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
-125.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
-126.Wait For Pageload,wait,3000,
-127. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
-128. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
-129. Click Agree,tap,,"mobile.driver.agree_continue.btn"
-130. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
-131. Enter OTP,type,123456,"mobile.driver.edit_text.input"
-132. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"</t>
+77.Click Submit,click,,"mobile.driver.bank_details.submit_btn"
+78.Wait For Logout,wait_until_visible,"mobile.drivers.after_upload_doc.logout_btn"
+79.Click Logout,tap,,"mobile.drivers.after_upload_doc.logout_btn"
+80.Click Confirm Logout,tap,,"mobile.drivers.after_upload_doc.logout_confirm_btn"
+81.Reload Driver App Completely,reload_app,driver,
+82.Load Admin App,switch_to,web,
+83.Wait For Dashboard,wait_until_visible,,"web.global.menu.dashboard"
+84.Click Dashboard Icon,click,,"web.global.menu.dashboard"
+85.Click drivers menu,click,,"admin.drivers.menu.icon"
+86.Click Pending Documents,click,,"admin.drivers.pending_docs.link"
+87.Filter by Name,type,{driverName},"admin.drivers.name_filter.input"
+98.Scroll Grid,tab,7,"admin.drivers.name_filter.input"
+89. Click Doc Icon,click,,"admin.drivers.docs.icon"
+90. Wait For Required Documents,wait_until_visible,,"admin.drivers.required_docs.header"
+91. FilterDocumet List,type,Driving Licence,"admin.drivers.docs_filter.input"
+92. Click Approve Driver,click,,"admin.drivers.docs.approval"
+93. Wait For Updated Successfully,wait_until_visible,,"web.global.toast.updated"
+94. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+95. Click drivers menu,click,,"admin.drivers.menu.icon"
+96. Click UnApproved Drivers,click,,"admin.drivers.unapproved_docs.link"
+97.Wait For load,wait,3000,
+98.Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
+99.Scroll Grid,tab,10,"admin.drivers.name_filter.input"
+100.Click Eye Icon,click,,"admin.drivers.unapproved_driver.eye_icon"
+101.Wait For Data,wait,3000,
+102.Click Close Button,click,,"admin.drivers.unapproved_driver.eye_icon.close_btn"
+103.Click ThumbsUp For Approve,click,,"admin.drivers.unapproved_driver.thumbs_up"
+104.Wait For Toast,wait,3000,
+105. Click Dashboard Icon,click,,"web.global.menu.dashboard"
+106.Click drivers menu,click,,"admin.drivers.menu.icon"
+107.Click Approved Drivers,click,,"admin.drivers.approved_docs.link"
+108.Wait For Approved Drivers List,wait_until_visible,,"admin.drivers.approved_page.header"
+109. Filter Approved Driver,type,{driverName},"admin.drivers.name_filter.input"
+110.Load Driver App,switch_to,driver,
+111.Wait For Notification,wait_until_visible,,"mobile.driver.permission_allow.btn"
+112.Click Allow Notification,tap,,"mobile.driver.permission_allow.btn"
+113.Click Agree,tap,,"mobile.driver.agree.btn"
+114.Click Get Started,tap,,"mobile.driver.get_started.btn"
+115.Click Next,tap,,"mobile.driver.next.btn"
+116.Click Mobile Number,tap,,"mobile.driver.mobile_number_field.btn"
+117.Click Close,tap,,"mobile.driver.cancel.btn"
+118.Enter Mobile Number,type,{driverNumber},"mobile.driver.edit_text.input"
+119.Wait for Continue,wait_until_visible,,"mobile.driver.continue.btn"
+120.Click Continue,tap,,"mobile.driver.continue.btn"
+121.Enter OTP,type,123456,"mobile.driver.edit_text.input"
+122.Click Allow Location,tap,,"mobile.driver.location_allow.btn"
+123.Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"
+124.Wait For Pageload,wait,3000,
+125. Click Select All Agree,tap,,"mobile.driver.independent_contractor.checkbox_Select_All"
+126. Wait for Agree,wait_until_visible,,"mobile.driver.agree_continue.btn"
+127. Click Agree,tap,,"mobile.driver.agree_continue.btn"
+128. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
+129. Enter OTP,type,123456,"mobile.driver.edit_text.input"
+130. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
110th Commit: Epic Nine And Eleven Completed
</commit_message>
<xml_diff>
--- a/EPIC_0002_Driver_Onboarding.xlsx
+++ b/EPIC_0002_Driver_Onboarding.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D11E450-966B-4F26-B836-A88833BBF920}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE9727B-01E1-4C37-83DC-CBCBC9FD2F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -311,9 +311,6 @@
   </si>
   <si>
     <t>Driver Onboarding</t>
-  </si>
-  <si>
-    <t>TC_RG_01_Driver_Onboarding</t>
   </si>
   <si>
     <t>This test case validates the end-to-end registration, verification, document approval, and login workflow for a new driver. It covers onboarding the driver via the mobile app by submitting personal details, capturing profile and vehicle images, selecting service parameters, uploading required compliance documents like a driving license with an expiry date, and configuring banking information. It then verifies the admin review lifecycle by logging into the Super Admin portal, filtering the pending application, approving the submitted driving license, and confirming the driver's transition to the approved drivers list. Finally, it verifies that the approved driver can re-authenticate via OTP on the mobile app and successfully access the driver dashboard with location permissions enabled.</t>
@@ -686,6 +683,9 @@
 128. Wait For OTP,wait_until_visible,,"mobile.driver.edit_text.input"
 129. Enter OTP,type,123456,"mobile.driver.edit_text.input"
 130. Wait For Driver App,wait_until_visible,,"mobile.driver.app_header.label"</t>
+  </si>
+  <si>
+    <t>TC_RG_02_Driver_Onboarding</t>
   </si>
 </sst>
 </file>
@@ -1187,25 +1187,25 @@
         <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>